<commit_message>
Update price, config and deal data
</commit_message>
<xml_diff>
--- a/config_sets.xlsx
+++ b/config_sets.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -747,28 +747,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>11508</t>
+          <t>21338</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Marguerites</t>
+          <t>La maison en A</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt515cd2564f9b2dcf/11508_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt2b163a472ef2e61f/21338.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/11508</t>
+          <t>https://www.lego.com/fr-fr/product/21338</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -779,28 +779,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11509</t>
+          <t>21365</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cactus fleuri</t>
+          <t>Les oiseaux amoureux</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>482</t>
+          <t>750</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt05c278dbcfaa4871/11509_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt859e843a3f8c5af9/21365_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/11509</t>
+          <t>https://www.lego.com/fr-fr/product/21365</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -811,28 +811,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>21338</t>
+          <t>31218</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>La maison en A</t>
+          <t>Les cerisiers en fleurs</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt2b163a472ef2e61f/21338.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt3f6cace2ff7687c6/31218_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/21338</t>
+          <t>https://www.lego.com/fr-fr/product/31218</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -843,28 +843,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>21365</t>
+          <t>31378</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Les oiseaux amoureux</t>
+          <t>Le télescope d’exploration spatiale</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>278</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt859e843a3f8c5af9/21365_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt71fe323b45263a78/31378_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/21365</t>
+          <t>https://www.lego.com/fr-fr/product/31378</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -875,28 +875,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>31218</t>
+          <t>31379</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Les cerisiers en fleurs</t>
+          <t>Le dinosaure féroce</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>283</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt3f6cace2ff7687c6/31218_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt94ad0e9878a39d0a/31379_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/31218</t>
+          <t>https://www.lego.com/fr-fr/product/31379</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -907,28 +907,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31378</t>
+          <t>31384</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Le télescope d’exploration spatiale</t>
+          <t>Animaux sauvages : le colibri coloré</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>312</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt71fe323b45263a78/31378_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blta735df411e869f69/31384_Prod_Crop.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/31378</t>
+          <t>https://www.lego.com/fr-fr/product/31384</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -939,28 +939,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31379</t>
+          <t>31385</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Le dinosaure féroce</t>
+          <t>Animaux marins : les beaux dauphins</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>283</t>
+          <t>542</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt94ad0e9878a39d0a/31379_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltbf6cbcbb8ff1610b/31385_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/31379</t>
+          <t>https://www.lego.com/fr-fr/product/31385</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -971,28 +971,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>31384</t>
+          <t>40957</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Animaux sauvages : le colibri coloré</t>
+          <t>La couronne printanière</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>747</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blta735df411e869f69/31384_Prod_Crop.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltd979e8936ef8f4e8/40957_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/31384</t>
+          <t>https://www.lego.com/fr-fr/product/40957</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1003,28 +1003,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>31385</t>
+          <t>42222</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Animaux marins : les beaux dauphins</t>
+          <t>Hypercar Bugatti Chiron Pur Sport</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>542</t>
+          <t>771</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltbf6cbcbb8ff1610b/31385_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt0a9009b95130ef89/42222_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/31385</t>
+          <t>https://www.lego.com/fr-fr/product/42222</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1035,28 +1035,28 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>40957</t>
+          <t>42227</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La couronne printanière</t>
+          <t>SUV Jeep® Wrangler Rubicon</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>747</t>
+          <t>723</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltd979e8936ef8f4e8/40957_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt8f7d3695517d3132/42227_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/40957</t>
+          <t>https://www.lego.com/fr-fr/product/42227</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1067,28 +1067,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>42222</t>
+          <t>43281</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hypercar Bugatti Chiron Pur Sport</t>
+          <t>Le château de glace et la piste enneigée d’Elsa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>216</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt0a9009b95130ef89/42222_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt3c56a41db2717b7b/43281_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/42222</t>
+          <t>https://www.lego.com/fr-fr/product/43281</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1099,28 +1099,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>42227</t>
+          <t>43287</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SUV Jeep® Wrangler Rubicon</t>
+          <t>Le pique-nique d’Olaf et Bruni</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>723</t>
+          <t>478</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt8f7d3695517d3132/42227_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt9bcf160a34a7c824/43287_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/42227</t>
+          <t>https://www.lego.com/fr-fr/product/43287</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1131,28 +1131,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>43281</t>
+          <t>45200</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Le château de glace et la piste enneigée d’Elsa</t>
+          <t>Kit de science Mission lunaire</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>519</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt3c56a41db2717b7b/43281_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltf7b7ce8f03c1660e/bltb54bf9af8b6f95a9-45200_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/43281</t>
+          <t>https://www.lego.com/fr-fr/product/45200</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1163,28 +1163,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>43287</t>
+          <t>75423</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Le pique-nique d’Olaf et Bruni</t>
+          <t>SMART Play™ : le X-Wing™ Red Five de Luke</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>581</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt9bcf160a34a7c824/43287_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt5083a28189d02095/75423_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/43287</t>
+          <t>https://www.lego.com/fr-fr/product/75423</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1195,28 +1195,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>45200</t>
+          <t>75440</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kit de science Mission lunaire</t>
+          <t>AT-AT™</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>519</t>
+          <t>525</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltf7b7ce8f03c1660e/bltb54bf9af8b6f95a9-45200_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blt26f813f1a1f499c6/75440_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/45200</t>
+          <t>https://www.lego.com/fr-fr/product/75440</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1227,28 +1227,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>75423</t>
+          <t>77256</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SMART Play™ : le X-Wing™ Red Five de Luke</t>
+          <t>La machine à remonter le temps de Retour vers le futur</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>357</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt5083a28189d02095/75423_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltcf1faba2d5f4a688/77256_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/75423</t>
+          <t>https://www.lego.com/fr-fr/product/77256</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1256,70 +1256,6 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>75440</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>AT-AT™</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>525</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blt26f813f1a1f499c6/75440_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>https://www.lego.com/fr-fr/product/75440</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>77256</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>La machine à remonter le temps de Retour vers le futur</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>357</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltcf1faba2d5f4a688/77256_Prod_en-gb.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://www.lego.com/fr-fr/product/77256</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>